<commit_message>
data(eur): daily refresh 2026-09-14T15:17Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="198" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="200" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -684,6 +684,12 @@
   </si>
   <si>
     <t>87</t>
+  </si>
+  <si>
+    <t>88</t>
+  </si>
+  <si>
+    <t>DE000BU0E451</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1127,7 +1133,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S167"/>
+  <dimension ref="A1:S169"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -9656,108 +9662,222 @@
       </c>
     </row>
     <row r="156" spans="1:19">
-      <c r="A156" s="50" t="s">
+      <c r="A156" s="36" t="s">
         <v>184</v>
       </c>
-      <c r="B156" s="48"/>
-      <c r="C156" s="48"/>
-      <c r="D156" s="48"/>
-      <c r="E156" s="48"/>
-      <c r="F156" s="48"/>
-      <c r="G156" s="49"/>
-      <c r="H156" s="52">
-        <v>388000</v>
-      </c>
-      <c r="I156" s="51"/>
-      <c r="J156" s="51"/>
-      <c r="K156" s="52">
-        <v>526645</v>
-      </c>
-      <c r="L156" s="52">
-        <v>308959</v>
-      </c>
-      <c r="M156" s="52">
-        <v>217686</v>
-      </c>
-      <c r="N156" s="53">
-        <v>305209.43</v>
-      </c>
-      <c r="O156" s="47"/>
-      <c r="P156" s="48"/>
-      <c r="Q156" s="48"/>
-      <c r="R156" s="49"/>
-      <c r="S156" s="54">
-        <v>1.724252517361</v>
-      </c>
-    </row>
-    <row r="157" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A157" s="21" t="s">
+      <c r="B156" s="37">
+        <v>46279</v>
+      </c>
+      <c r="C156" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D156" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E156" s="35"/>
+      <c r="F156" s="37">
+        <v>46463</v>
+      </c>
+      <c r="G156" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H156" s="39">
+        <v>2000</v>
+      </c>
+      <c r="I156" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J156" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K156" s="39">
+        <v>3170</v>
+      </c>
+      <c r="L156" s="39">
+        <v>2605</v>
+      </c>
+      <c r="M156" s="39">
+        <v>565</v>
+      </c>
+      <c r="N156" s="40">
+        <v>1825</v>
+      </c>
+      <c r="O156" s="41">
+        <v>98.61698</v>
+      </c>
+      <c r="P156" s="42">
+        <v>98.61993</v>
+      </c>
+      <c r="Q156" s="43">
+        <v>2.768</v>
+      </c>
+      <c r="R156" s="40">
+        <v>175</v>
+      </c>
+      <c r="S156" s="44">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="157" spans="1:19">
+      <c r="A157" s="36" t="s">
+        <v>184</v>
+      </c>
+      <c r="B157" s="37">
+        <v>46279</v>
+      </c>
+      <c r="C157" s="36" t="s">
+        <v>185</v>
+      </c>
+      <c r="D157" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E157" s="35"/>
+      <c r="F157" s="37">
+        <v>46645</v>
+      </c>
+      <c r="G157" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H157" s="39">
+        <v>4000</v>
+      </c>
+      <c r="I157" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="J157" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K157" s="39">
+        <v>6565</v>
+      </c>
+      <c r="L157" s="39">
+        <v>4360</v>
+      </c>
+      <c r="M157" s="39">
+        <v>2205</v>
+      </c>
+      <c r="N157" s="40">
+        <v>3650</v>
+      </c>
+      <c r="O157" s="41">
+        <v>96.99029</v>
+      </c>
+      <c r="P157" s="42">
+        <v>96.9941</v>
+      </c>
+      <c r="Q157" s="43">
+        <v>3.065</v>
+      </c>
+      <c r="R157" s="40">
+        <v>350</v>
+      </c>
+      <c r="S157" s="44">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="158" spans="1:19">
+      <c r="A158" s="50" t="s">
+        <v>186</v>
+      </c>
+      <c r="B158" s="48"/>
+      <c r="C158" s="48"/>
+      <c r="D158" s="48"/>
+      <c r="E158" s="48"/>
+      <c r="F158" s="48"/>
+      <c r="G158" s="49"/>
+      <c r="H158" s="52">
+        <v>394000</v>
+      </c>
+      <c r="I158" s="51"/>
+      <c r="J158" s="51"/>
+      <c r="K158" s="52">
+        <v>536380</v>
+      </c>
+      <c r="L158" s="52">
+        <v>315924</v>
+      </c>
+      <c r="M158" s="52">
+        <v>220456</v>
+      </c>
+      <c r="N158" s="53">
+        <v>310684.43</v>
+      </c>
+      <c r="O158" s="47"/>
+      <c r="P158" s="48"/>
+      <c r="Q158" s="48"/>
+      <c r="R158" s="49"/>
+      <c r="S158" s="54">
+        <v>1.724999955742</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A159" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:2">
-      <c r="A158" s="22" t="s">
+    <row r="160" spans="1:2">
+      <c r="A160" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B158" s="22" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="159" spans="1:1">
-      <c r="A159" s="22" t="s">
+      <c r="B160" s="22" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1">
+      <c r="A161" s="22" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2">
-      <c r="A160" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="B160" s="26" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="B162" s="22" t="s">
+      <c r="B162" s="26" t="s">
         <v>189</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2">
-      <c r="A163" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="B163" s="22" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="23" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B164" s="22" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B165" s="22" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="23" t="s">
         <v>194</v>
       </c>
-      <c r="B165" s="22" t="s">
+      <c r="B166" s="22" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="166" spans="1:2">
-      <c r="A166" s="24" t="s">
+    <row r="167" spans="1:2">
+      <c r="A167" s="23" t="s">
         <v>196</v>
       </c>
-      <c r="B166" s="22" t="s">
+      <c r="B167" s="22" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="167" spans="1:1">
-      <c r="A167" s="25" t="s">
+    <row r="168" spans="1:2">
+      <c r="A168" s="24" t="s">
+        <v>198</v>
+      </c>
+      <c r="B168" s="22" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1">
+      <c r="A169" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -9767,16 +9887,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A156:G156"/>
-    <mergeCell ref="O156:R156"/>
-    <mergeCell ref="B158:R158"/>
-    <mergeCell ref="A160:A161"/>
-    <mergeCell ref="B160:R161"/>
-    <mergeCell ref="B162:R162"/>
-    <mergeCell ref="B163:R163"/>
+    <mergeCell ref="A158:G158"/>
+    <mergeCell ref="O158:R158"/>
+    <mergeCell ref="B160:R160"/>
+    <mergeCell ref="A162:A163"/>
+    <mergeCell ref="B162:R163"/>
     <mergeCell ref="B164:R164"/>
     <mergeCell ref="B165:R165"/>
     <mergeCell ref="B166:R166"/>
+    <mergeCell ref="B167:R167"/>
+    <mergeCell ref="B168:R168"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-09-15T13:54Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="200" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -690,6 +690,9 @@
   </si>
   <si>
     <t>DE000BU0E451</t>
+  </si>
+  <si>
+    <t>89</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1133,7 +1136,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S169"/>
+  <dimension ref="A1:S170"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -9776,108 +9779,167 @@
       </c>
     </row>
     <row r="158" spans="1:19">
-      <c r="A158" s="50" t="s">
+      <c r="A158" s="36" t="s">
         <v>186</v>
       </c>
-      <c r="B158" s="48"/>
-      <c r="C158" s="48"/>
-      <c r="D158" s="48"/>
-      <c r="E158" s="48"/>
-      <c r="F158" s="48"/>
-      <c r="G158" s="49"/>
-      <c r="H158" s="52">
-        <v>394000</v>
-      </c>
-      <c r="I158" s="51"/>
-      <c r="J158" s="51"/>
-      <c r="K158" s="52">
-        <v>536380</v>
-      </c>
-      <c r="L158" s="52">
-        <v>315924</v>
-      </c>
-      <c r="M158" s="52">
-        <v>220456</v>
-      </c>
-      <c r="N158" s="53">
-        <v>310684.43</v>
-      </c>
-      <c r="O158" s="47"/>
-      <c r="P158" s="48"/>
-      <c r="Q158" s="48"/>
-      <c r="R158" s="49"/>
-      <c r="S158" s="54">
-        <v>1.724999955742</v>
-      </c>
-    </row>
-    <row r="159" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A159" s="21" t="s">
+      <c r="B158" s="37">
+        <v>46280</v>
+      </c>
+      <c r="C158" s="36" t="s">
+        <v>162</v>
+      </c>
+      <c r="D158" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="E158" s="45">
+        <v>0.027</v>
+      </c>
+      <c r="F158" s="37">
+        <v>47009</v>
+      </c>
+      <c r="G158" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="H158" s="39">
+        <v>5000</v>
+      </c>
+      <c r="I158" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J158" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="K158" s="39">
+        <v>4816</v>
+      </c>
+      <c r="L158" s="39">
+        <v>2668</v>
+      </c>
+      <c r="M158" s="39">
+        <v>2148</v>
+      </c>
+      <c r="N158" s="40">
+        <v>3816.88</v>
+      </c>
+      <c r="O158" s="41">
+        <v>98.9</v>
+      </c>
+      <c r="P158" s="43">
+        <v>98.906</v>
+      </c>
+      <c r="Q158" s="40">
+        <v>3.27</v>
+      </c>
+      <c r="R158" s="40">
+        <v>1183.12</v>
+      </c>
+      <c r="S158" s="44">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="159" spans="1:19">
+      <c r="A159" s="50" t="s">
+        <v>187</v>
+      </c>
+      <c r="B159" s="48"/>
+      <c r="C159" s="48"/>
+      <c r="D159" s="48"/>
+      <c r="E159" s="48"/>
+      <c r="F159" s="48"/>
+      <c r="G159" s="49"/>
+      <c r="H159" s="52">
+        <v>399000</v>
+      </c>
+      <c r="I159" s="51"/>
+      <c r="J159" s="51"/>
+      <c r="K159" s="52">
+        <v>541196</v>
+      </c>
+      <c r="L159" s="52">
+        <v>318592</v>
+      </c>
+      <c r="M159" s="52">
+        <v>222604</v>
+      </c>
+      <c r="N159" s="53">
+        <v>314501.31</v>
+      </c>
+      <c r="O159" s="47"/>
+      <c r="P159" s="48"/>
+      <c r="Q159" s="48"/>
+      <c r="R159" s="49"/>
+      <c r="S159" s="54">
+        <v>1.719842031818</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A160" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:2">
-      <c r="A160" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="B160" s="22" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="161" spans="1:1">
+    <row r="161" spans="1:2">
       <c r="A161" s="22" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="162" spans="1:2">
-      <c r="A162" s="23" t="s">
+      <c r="B161" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="B162" s="26" t="s">
+    </row>
+    <row r="162" spans="1:1">
+      <c r="A162" s="22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="23" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="164" spans="1:2">
-      <c r="A164" s="23" t="s">
+      <c r="B163" s="26" t="s">
         <v>190</v>
-      </c>
-      <c r="B164" s="22" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="B165" s="22" t="s">
         <v>192</v>
-      </c>
-      <c r="B165" s="22" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="B166" s="22" t="s">
         <v>194</v>
-      </c>
-      <c r="B166" s="22" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="B167" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="B167" s="22" t="s">
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="23" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="168" spans="1:2">
-      <c r="A168" s="24" t="s">
+      <c r="B168" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="B168" s="22" t="s">
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="24" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="169" spans="1:1">
-      <c r="A169" s="25" t="s">
+      <c r="B169" s="22" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1">
+      <c r="A170" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -9887,16 +9949,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A158:G158"/>
-    <mergeCell ref="O158:R158"/>
-    <mergeCell ref="B160:R160"/>
-    <mergeCell ref="A162:A163"/>
-    <mergeCell ref="B162:R163"/>
-    <mergeCell ref="B164:R164"/>
+    <mergeCell ref="A159:G159"/>
+    <mergeCell ref="O159:R159"/>
+    <mergeCell ref="B161:R161"/>
+    <mergeCell ref="A163:A164"/>
+    <mergeCell ref="B163:R164"/>
     <mergeCell ref="B165:R165"/>
     <mergeCell ref="B166:R166"/>
     <mergeCell ref="B167:R167"/>
     <mergeCell ref="B168:R168"/>
+    <mergeCell ref="B169:R169"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-09-16T13:46Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="202" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -693,6 +693,9 @@
   </si>
   <si>
     <t>89</t>
+  </si>
+  <si>
+    <t>90</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1136,7 +1139,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S170"/>
+  <dimension ref="A1:S172"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -9838,108 +9841,226 @@
       </c>
     </row>
     <row r="159" spans="1:19">
-      <c r="A159" s="50" t="s">
+      <c r="A159" s="36" t="s">
         <v>187</v>
       </c>
-      <c r="B159" s="48"/>
-      <c r="C159" s="48"/>
-      <c r="D159" s="48"/>
-      <c r="E159" s="48"/>
-      <c r="F159" s="48"/>
-      <c r="G159" s="49"/>
-      <c r="H159" s="52">
-        <v>399000</v>
-      </c>
-      <c r="I159" s="51"/>
-      <c r="J159" s="51"/>
-      <c r="K159" s="52">
-        <v>541196</v>
-      </c>
-      <c r="L159" s="52">
-        <v>318592</v>
-      </c>
-      <c r="M159" s="52">
-        <v>222604</v>
-      </c>
-      <c r="N159" s="53">
-        <v>314501.31</v>
-      </c>
-      <c r="O159" s="47"/>
-      <c r="P159" s="48"/>
-      <c r="Q159" s="48"/>
-      <c r="R159" s="49"/>
-      <c r="S159" s="54">
-        <v>1.719842031818</v>
-      </c>
-    </row>
-    <row r="160" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A160" s="21" t="s">
+      <c r="B159" s="37">
+        <v>46281</v>
+      </c>
+      <c r="C159" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="D159" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E159" s="45">
+        <v>0.034</v>
+      </c>
+      <c r="F159" s="37">
+        <v>53827</v>
+      </c>
+      <c r="G159" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="H159" s="39">
+        <v>1000</v>
+      </c>
+      <c r="I159" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J159" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K159" s="39">
+        <v>2110</v>
+      </c>
+      <c r="L159" s="39">
+        <v>1177</v>
+      </c>
+      <c r="M159" s="39">
+        <v>933</v>
+      </c>
+      <c r="N159" s="40">
+        <v>863.82</v>
+      </c>
+      <c r="O159" s="41">
+        <v>93.19</v>
+      </c>
+      <c r="P159" s="40">
+        <v>93.21</v>
+      </c>
+      <c r="Q159" s="40">
+        <v>3.88</v>
+      </c>
+      <c r="R159" s="40">
+        <v>136.18</v>
+      </c>
+      <c r="S159" s="44">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="160" spans="1:19">
+      <c r="A160" s="36" t="s">
+        <v>187</v>
+      </c>
+      <c r="B160" s="37">
+        <v>46281</v>
+      </c>
+      <c r="C160" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="D160" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E160" s="45">
+        <v>0.029</v>
+      </c>
+      <c r="F160" s="37">
+        <v>57207</v>
+      </c>
+      <c r="G160" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="H160" s="39">
+        <v>1500</v>
+      </c>
+      <c r="I160" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J160" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K160" s="39">
+        <v>3049</v>
+      </c>
+      <c r="L160" s="39">
+        <v>1348</v>
+      </c>
+      <c r="M160" s="39">
+        <v>1701</v>
+      </c>
+      <c r="N160" s="40">
+        <v>1257.41</v>
+      </c>
+      <c r="O160" s="41">
+        <v>82.49</v>
+      </c>
+      <c r="P160" s="40">
+        <v>82.57</v>
+      </c>
+      <c r="Q160" s="40">
+        <v>3.9</v>
+      </c>
+      <c r="R160" s="40">
+        <v>242.59</v>
+      </c>
+      <c r="S160" s="44">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="161" spans="1:19">
+      <c r="A161" s="50" t="s">
+        <v>188</v>
+      </c>
+      <c r="B161" s="48"/>
+      <c r="C161" s="48"/>
+      <c r="D161" s="48"/>
+      <c r="E161" s="48"/>
+      <c r="F161" s="48"/>
+      <c r="G161" s="49"/>
+      <c r="H161" s="52">
+        <v>401500</v>
+      </c>
+      <c r="I161" s="51"/>
+      <c r="J161" s="51"/>
+      <c r="K161" s="52">
+        <v>546355</v>
+      </c>
+      <c r="L161" s="52">
+        <v>321117</v>
+      </c>
+      <c r="M161" s="52">
+        <v>225238</v>
+      </c>
+      <c r="N161" s="53">
+        <v>316622.54</v>
+      </c>
+      <c r="O161" s="47"/>
+      <c r="P161" s="48"/>
+      <c r="Q161" s="48"/>
+      <c r="R161" s="49"/>
+      <c r="S161" s="54">
+        <v>1.724398787275</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A162" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:2">
-      <c r="A161" s="22" t="s">
+    <row r="163" spans="1:2">
+      <c r="A163" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B161" s="22" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="162" spans="1:1">
-      <c r="A162" s="22" t="s">
+      <c r="B163" s="22" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1">
+      <c r="A164" s="22" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2">
-      <c r="A163" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="B163" s="26" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="B165" s="26" t="s">
         <v>191</v>
-      </c>
-      <c r="B165" s="22" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2">
-      <c r="A166" s="23" t="s">
-        <v>193</v>
-      </c>
-      <c r="B166" s="22" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="23" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B167" s="22" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="B168" s="22" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="B169" s="22" t="s">
         <v>197</v>
       </c>
-      <c r="B168" s="22" t="s">
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="23" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="169" spans="1:2">
-      <c r="A169" s="24" t="s">
+      <c r="B170" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="B169" s="22" t="s">
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="24" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="170" spans="1:1">
-      <c r="A170" s="25" t="s">
+      <c r="B171" s="22" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1">
+      <c r="A172" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -9949,16 +10070,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A159:G159"/>
-    <mergeCell ref="O159:R159"/>
-    <mergeCell ref="B161:R161"/>
-    <mergeCell ref="A163:A164"/>
-    <mergeCell ref="B163:R164"/>
-    <mergeCell ref="B165:R165"/>
-    <mergeCell ref="B166:R166"/>
+    <mergeCell ref="A161:G161"/>
+    <mergeCell ref="O161:R161"/>
+    <mergeCell ref="B163:R163"/>
+    <mergeCell ref="A165:A166"/>
+    <mergeCell ref="B165:R166"/>
     <mergeCell ref="B167:R167"/>
     <mergeCell ref="B168:R168"/>
     <mergeCell ref="B169:R169"/>
+    <mergeCell ref="B170:R170"/>
+    <mergeCell ref="B171:R171"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-09-21T15:22Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="202" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -696,6 +696,9 @@
   </si>
   <si>
     <t>90</t>
+  </si>
+  <si>
+    <t>91</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1139,7 +1142,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S172"/>
+  <dimension ref="A1:S174"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -9959,108 +9962,222 @@
       </c>
     </row>
     <row r="161" spans="1:19">
-      <c r="A161" s="50" t="s">
+      <c r="A161" s="36" t="s">
         <v>188</v>
       </c>
-      <c r="B161" s="48"/>
-      <c r="C161" s="48"/>
-      <c r="D161" s="48"/>
-      <c r="E161" s="48"/>
-      <c r="F161" s="48"/>
-      <c r="G161" s="49"/>
-      <c r="H161" s="52">
-        <v>401500</v>
-      </c>
-      <c r="I161" s="51"/>
-      <c r="J161" s="51"/>
-      <c r="K161" s="52">
-        <v>546355</v>
-      </c>
-      <c r="L161" s="52">
-        <v>321117</v>
-      </c>
-      <c r="M161" s="52">
-        <v>225238</v>
-      </c>
-      <c r="N161" s="53">
-        <v>316622.54</v>
-      </c>
-      <c r="O161" s="47"/>
-      <c r="P161" s="48"/>
-      <c r="Q161" s="48"/>
-      <c r="R161" s="49"/>
-      <c r="S161" s="54">
-        <v>1.724398787275</v>
-      </c>
-    </row>
-    <row r="162" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A162" s="21" t="s">
+      <c r="B161" s="37">
+        <v>46286</v>
+      </c>
+      <c r="C161" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="D161" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E161" s="35"/>
+      <c r="F161" s="37">
+        <v>46435</v>
+      </c>
+      <c r="G161" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H161" s="39">
+        <v>3000</v>
+      </c>
+      <c r="I161" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J161" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K161" s="39">
+        <v>5035</v>
+      </c>
+      <c r="L161" s="39">
+        <v>3610</v>
+      </c>
+      <c r="M161" s="39">
+        <v>1425</v>
+      </c>
+      <c r="N161" s="40">
+        <v>2930</v>
+      </c>
+      <c r="O161" s="41">
+        <v>98.90633</v>
+      </c>
+      <c r="P161" s="42">
+        <v>98.90912</v>
+      </c>
+      <c r="Q161" s="43">
+        <v>2.701</v>
+      </c>
+      <c r="R161" s="40">
+        <v>70</v>
+      </c>
+      <c r="S161" s="44">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="162" spans="1:19">
+      <c r="A162" s="36" t="s">
+        <v>188</v>
+      </c>
+      <c r="B162" s="37">
+        <v>46286</v>
+      </c>
+      <c r="C162" s="36" t="s">
+        <v>175</v>
+      </c>
+      <c r="D162" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E162" s="35"/>
+      <c r="F162" s="37">
+        <v>46617</v>
+      </c>
+      <c r="G162" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H162" s="39">
+        <v>2000</v>
+      </c>
+      <c r="I162" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J162" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K162" s="39">
+        <v>6287</v>
+      </c>
+      <c r="L162" s="39">
+        <v>4525</v>
+      </c>
+      <c r="M162" s="39">
+        <v>1762</v>
+      </c>
+      <c r="N162" s="40">
+        <v>1985.8</v>
+      </c>
+      <c r="O162" s="41">
+        <v>97.34448</v>
+      </c>
+      <c r="P162" s="42">
+        <v>97.34795</v>
+      </c>
+      <c r="Q162" s="43">
+        <v>2.981</v>
+      </c>
+      <c r="R162" s="40">
+        <v>14.2</v>
+      </c>
+      <c r="S162" s="44">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="163" spans="1:19">
+      <c r="A163" s="50" t="s">
+        <v>189</v>
+      </c>
+      <c r="B163" s="48"/>
+      <c r="C163" s="48"/>
+      <c r="D163" s="48"/>
+      <c r="E163" s="48"/>
+      <c r="F163" s="48"/>
+      <c r="G163" s="49"/>
+      <c r="H163" s="52">
+        <v>406500</v>
+      </c>
+      <c r="I163" s="51"/>
+      <c r="J163" s="51"/>
+      <c r="K163" s="52">
+        <v>557677</v>
+      </c>
+      <c r="L163" s="52">
+        <v>329252</v>
+      </c>
+      <c r="M163" s="52">
+        <v>228425</v>
+      </c>
+      <c r="N163" s="53">
+        <v>321538.34</v>
+      </c>
+      <c r="O163" s="47"/>
+      <c r="P163" s="48"/>
+      <c r="Q163" s="48"/>
+      <c r="R163" s="49"/>
+      <c r="S163" s="54">
+        <v>1.733289672391</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A164" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:2">
-      <c r="A163" s="22" t="s">
+    <row r="165" spans="1:2">
+      <c r="A165" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B163" s="22" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="164" spans="1:1">
-      <c r="A164" s="22" t="s">
+      <c r="B165" s="22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1">
+      <c r="A166" s="22" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2">
-      <c r="A165" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="B165" s="26" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="B167" s="26" t="s">
         <v>192</v>
-      </c>
-      <c r="B167" s="22" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="168" spans="1:2">
-      <c r="A168" s="23" t="s">
-        <v>194</v>
-      </c>
-      <c r="B168" s="22" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="23" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B169" s="22" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="B170" s="22" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="B171" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="B170" s="22" t="s">
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="23" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="171" spans="1:2">
-      <c r="A171" s="24" t="s">
+      <c r="B172" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="B171" s="22" t="s">
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="24" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="172" spans="1:1">
-      <c r="A172" s="25" t="s">
+      <c r="B173" s="22" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1">
+      <c r="A174" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -10070,16 +10187,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A161:G161"/>
-    <mergeCell ref="O161:R161"/>
-    <mergeCell ref="B163:R163"/>
-    <mergeCell ref="A165:A166"/>
-    <mergeCell ref="B165:R166"/>
-    <mergeCell ref="B167:R167"/>
-    <mergeCell ref="B168:R168"/>
+    <mergeCell ref="A163:G163"/>
+    <mergeCell ref="O163:R163"/>
+    <mergeCell ref="B165:R165"/>
+    <mergeCell ref="A167:A168"/>
+    <mergeCell ref="B167:R168"/>
     <mergeCell ref="B169:R169"/>
     <mergeCell ref="B170:R170"/>
     <mergeCell ref="B171:R171"/>
+    <mergeCell ref="B172:R172"/>
+    <mergeCell ref="B173:R173"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-09-22T13:42Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="204" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -699,6 +699,9 @@
   </si>
   <si>
     <t>91</t>
+  </si>
+  <si>
+    <t>92</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1142,7 +1145,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S174"/>
+  <dimension ref="A1:S175"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -10076,108 +10079,167 @@
       </c>
     </row>
     <row r="163" spans="1:19">
-      <c r="A163" s="50" t="s">
+      <c r="A163" s="36" t="s">
         <v>189</v>
       </c>
-      <c r="B163" s="48"/>
-      <c r="C163" s="48"/>
-      <c r="D163" s="48"/>
-      <c r="E163" s="48"/>
-      <c r="F163" s="48"/>
-      <c r="G163" s="49"/>
-      <c r="H163" s="52">
-        <v>406500</v>
-      </c>
-      <c r="I163" s="51"/>
-      <c r="J163" s="51"/>
-      <c r="K163" s="52">
-        <v>557677</v>
-      </c>
-      <c r="L163" s="52">
-        <v>329252</v>
-      </c>
-      <c r="M163" s="52">
-        <v>228425</v>
-      </c>
-      <c r="N163" s="53">
-        <v>321538.34</v>
-      </c>
-      <c r="O163" s="47"/>
-      <c r="P163" s="48"/>
-      <c r="Q163" s="48"/>
-      <c r="R163" s="49"/>
-      <c r="S163" s="54">
-        <v>1.733289672391</v>
-      </c>
-    </row>
-    <row r="164" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A164" s="21" t="s">
+      <c r="B163" s="37">
+        <v>46287</v>
+      </c>
+      <c r="C163" s="36" t="s">
+        <v>166</v>
+      </c>
+      <c r="D163" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="E163" s="45">
+        <v>0.029</v>
+      </c>
+      <c r="F163" s="37">
+        <v>48129</v>
+      </c>
+      <c r="G163" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="H163" s="39">
+        <v>5000</v>
+      </c>
+      <c r="I163" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J163" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="K163" s="39">
+        <v>4530</v>
+      </c>
+      <c r="L163" s="39">
+        <v>2470</v>
+      </c>
+      <c r="M163" s="39">
+        <v>2060</v>
+      </c>
+      <c r="N163" s="40">
+        <v>3735</v>
+      </c>
+      <c r="O163" s="41">
+        <v>98.23</v>
+      </c>
+      <c r="P163" s="40">
+        <v>98.24</v>
+      </c>
+      <c r="Q163" s="40">
+        <v>3.28</v>
+      </c>
+      <c r="R163" s="40">
+        <v>1265</v>
+      </c>
+      <c r="S163" s="44">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="164" spans="1:19">
+      <c r="A164" s="50" t="s">
+        <v>190</v>
+      </c>
+      <c r="B164" s="48"/>
+      <c r="C164" s="48"/>
+      <c r="D164" s="48"/>
+      <c r="E164" s="48"/>
+      <c r="F164" s="48"/>
+      <c r="G164" s="49"/>
+      <c r="H164" s="52">
+        <v>411500</v>
+      </c>
+      <c r="I164" s="51"/>
+      <c r="J164" s="51"/>
+      <c r="K164" s="52">
+        <v>562207</v>
+      </c>
+      <c r="L164" s="52">
+        <v>331722</v>
+      </c>
+      <c r="M164" s="52">
+        <v>230485</v>
+      </c>
+      <c r="N164" s="53">
+        <v>325273.34</v>
+      </c>
+      <c r="O164" s="47"/>
+      <c r="P164" s="48"/>
+      <c r="Q164" s="48"/>
+      <c r="R164" s="49"/>
+      <c r="S164" s="54">
+        <v>1.727166093599</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A165" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:2">
-      <c r="A165" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="B165" s="22" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="166" spans="1:1">
+    <row r="166" spans="1:2">
       <c r="A166" s="22" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="167" spans="1:2">
-      <c r="A167" s="23" t="s">
+      <c r="B166" s="22" t="s">
         <v>191</v>
       </c>
-      <c r="B167" s="26" t="s">
+    </row>
+    <row r="167" spans="1:1">
+      <c r="A167" s="22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="23" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="169" spans="1:2">
-      <c r="A169" s="23" t="s">
+      <c r="B168" s="26" t="s">
         <v>193</v>
-      </c>
-      <c r="B169" s="22" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="B170" s="22" t="s">
         <v>195</v>
-      </c>
-      <c r="B170" s="22" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="B171" s="22" t="s">
         <v>197</v>
-      </c>
-      <c r="B171" s="22" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B172" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="B172" s="22" t="s">
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="23" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="173" spans="1:2">
-      <c r="A173" s="24" t="s">
+      <c r="B173" s="22" t="s">
         <v>201</v>
       </c>
-      <c r="B173" s="22" t="s">
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="24" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="174" spans="1:1">
-      <c r="A174" s="25" t="s">
+      <c r="B174" s="22" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1">
+      <c r="A175" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -10187,16 +10249,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A163:G163"/>
-    <mergeCell ref="O163:R163"/>
-    <mergeCell ref="B165:R165"/>
-    <mergeCell ref="A167:A168"/>
-    <mergeCell ref="B167:R168"/>
-    <mergeCell ref="B169:R169"/>
+    <mergeCell ref="A164:G164"/>
+    <mergeCell ref="O164:R164"/>
+    <mergeCell ref="B166:R166"/>
+    <mergeCell ref="A168:A169"/>
+    <mergeCell ref="B168:R169"/>
     <mergeCell ref="B170:R170"/>
     <mergeCell ref="B171:R171"/>
     <mergeCell ref="B172:R172"/>
     <mergeCell ref="B173:R173"/>
+    <mergeCell ref="B174:R174"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-09-23T13:53Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="204" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -702,6 +702,9 @@
   </si>
   <si>
     <t>92</t>
+  </si>
+  <si>
+    <t>93</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1145,7 +1148,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S175"/>
+  <dimension ref="A1:S177"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -10138,108 +10141,226 @@
       </c>
     </row>
     <row r="164" spans="1:19">
-      <c r="A164" s="50" t="s">
+      <c r="A164" s="36" t="s">
         <v>190</v>
       </c>
-      <c r="B164" s="48"/>
-      <c r="C164" s="48"/>
-      <c r="D164" s="48"/>
-      <c r="E164" s="48"/>
-      <c r="F164" s="48"/>
-      <c r="G164" s="49"/>
-      <c r="H164" s="52">
-        <v>411500</v>
-      </c>
-      <c r="I164" s="51"/>
-      <c r="J164" s="51"/>
-      <c r="K164" s="52">
-        <v>562207</v>
-      </c>
-      <c r="L164" s="52">
-        <v>331722</v>
-      </c>
-      <c r="M164" s="52">
-        <v>230485</v>
-      </c>
-      <c r="N164" s="53">
-        <v>325273.34</v>
-      </c>
-      <c r="O164" s="47"/>
-      <c r="P164" s="48"/>
-      <c r="Q164" s="48"/>
-      <c r="R164" s="49"/>
-      <c r="S164" s="54">
-        <v>1.727166093599</v>
-      </c>
-    </row>
-    <row r="165" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A165" s="21" t="s">
+      <c r="B164" s="37">
+        <v>46288</v>
+      </c>
+      <c r="C164" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="D164" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E164" s="45">
+        <v>0.034</v>
+      </c>
+      <c r="F164" s="37">
+        <v>53827</v>
+      </c>
+      <c r="G164" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="H164" s="39">
+        <v>1000</v>
+      </c>
+      <c r="I164" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J164" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K164" s="39">
+        <v>1794</v>
+      </c>
+      <c r="L164" s="39">
+        <v>747</v>
+      </c>
+      <c r="M164" s="39">
+        <v>1047</v>
+      </c>
+      <c r="N164" s="40">
+        <v>869.74</v>
+      </c>
+      <c r="O164" s="41">
+        <v>94.52</v>
+      </c>
+      <c r="P164" s="40">
+        <v>94.53</v>
+      </c>
+      <c r="Q164" s="40">
+        <v>3.78</v>
+      </c>
+      <c r="R164" s="40">
+        <v>130.26</v>
+      </c>
+      <c r="S164" s="44">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:19">
+      <c r="A165" s="36" t="s">
+        <v>190</v>
+      </c>
+      <c r="B165" s="37">
+        <v>46288</v>
+      </c>
+      <c r="C165" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="D165" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E165" s="45">
+        <v>0.029</v>
+      </c>
+      <c r="F165" s="37">
+        <v>57207</v>
+      </c>
+      <c r="G165" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="H165" s="39">
+        <v>1000</v>
+      </c>
+      <c r="I165" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J165" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K165" s="39">
+        <v>1241</v>
+      </c>
+      <c r="L165" s="39">
+        <v>661</v>
+      </c>
+      <c r="M165" s="39">
+        <v>580</v>
+      </c>
+      <c r="N165" s="40">
+        <v>783.6</v>
+      </c>
+      <c r="O165" s="41">
+        <v>84.04</v>
+      </c>
+      <c r="P165" s="40">
+        <v>84.05</v>
+      </c>
+      <c r="Q165" s="40">
+        <v>3.8</v>
+      </c>
+      <c r="R165" s="40">
+        <v>216.4</v>
+      </c>
+      <c r="S165" s="44">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="166" spans="1:19">
+      <c r="A166" s="50" t="s">
+        <v>191</v>
+      </c>
+      <c r="B166" s="48"/>
+      <c r="C166" s="48"/>
+      <c r="D166" s="48"/>
+      <c r="E166" s="48"/>
+      <c r="F166" s="48"/>
+      <c r="G166" s="49"/>
+      <c r="H166" s="52">
+        <v>413500</v>
+      </c>
+      <c r="I166" s="51"/>
+      <c r="J166" s="51"/>
+      <c r="K166" s="52">
+        <v>565242</v>
+      </c>
+      <c r="L166" s="52">
+        <v>333130</v>
+      </c>
+      <c r="M166" s="52">
+        <v>232112</v>
+      </c>
+      <c r="N166" s="53">
+        <v>326926.68</v>
+      </c>
+      <c r="O166" s="47"/>
+      <c r="P166" s="48"/>
+      <c r="Q166" s="48"/>
+      <c r="R166" s="49"/>
+      <c r="S166" s="54">
+        <v>1.727853162672</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A167" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:2">
-      <c r="A166" s="22" t="s">
+    <row r="168" spans="1:2">
+      <c r="A168" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B166" s="22" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="167" spans="1:1">
-      <c r="A167" s="22" t="s">
+      <c r="B168" s="22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1">
+      <c r="A169" s="22" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="168" spans="1:2">
-      <c r="A168" s="23" t="s">
-        <v>192</v>
-      </c>
-      <c r="B168" s="26" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="B170" s="26" t="s">
         <v>194</v>
-      </c>
-      <c r="B170" s="22" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2">
-      <c r="A171" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="B171" s="22" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="23" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B172" s="22" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="B173" s="22" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="B174" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="B173" s="22" t="s">
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="23" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="174" spans="1:2">
-      <c r="A174" s="24" t="s">
+      <c r="B175" s="22" t="s">
         <v>202</v>
       </c>
-      <c r="B174" s="22" t="s">
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="24" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="175" spans="1:1">
-      <c r="A175" s="25" t="s">
+      <c r="B176" s="22" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1">
+      <c r="A177" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -10249,16 +10370,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A164:G164"/>
-    <mergeCell ref="O164:R164"/>
-    <mergeCell ref="B166:R166"/>
-    <mergeCell ref="A168:A169"/>
-    <mergeCell ref="B168:R169"/>
-    <mergeCell ref="B170:R170"/>
-    <mergeCell ref="B171:R171"/>
+    <mergeCell ref="A166:G166"/>
+    <mergeCell ref="O166:R166"/>
+    <mergeCell ref="B168:R168"/>
+    <mergeCell ref="A170:A171"/>
+    <mergeCell ref="B170:R171"/>
     <mergeCell ref="B172:R172"/>
     <mergeCell ref="B173:R173"/>
     <mergeCell ref="B174:R174"/>
+    <mergeCell ref="B175:R175"/>
+    <mergeCell ref="B176:R176"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-10-06T15:29Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="209" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -705,6 +705,18 @@
   </si>
   <si>
     <t>93</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>96</t>
+  </si>
+  <si>
+    <t>DE000BU22155</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1148,7 +1160,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S177"/>
+  <dimension ref="A1:S181"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -10259,108 +10271,340 @@
       </c>
     </row>
     <row r="166" spans="1:19">
-      <c r="A166" s="50" t="s">
+      <c r="A166" s="36" t="s">
         <v>191</v>
       </c>
-      <c r="B166" s="48"/>
-      <c r="C166" s="48"/>
-      <c r="D166" s="48"/>
-      <c r="E166" s="48"/>
-      <c r="F166" s="48"/>
-      <c r="G166" s="49"/>
-      <c r="H166" s="52">
-        <v>413500</v>
-      </c>
-      <c r="I166" s="51"/>
-      <c r="J166" s="51"/>
-      <c r="K166" s="52">
-        <v>565242</v>
-      </c>
-      <c r="L166" s="52">
-        <v>333130</v>
-      </c>
-      <c r="M166" s="52">
-        <v>232112</v>
-      </c>
-      <c r="N166" s="53">
-        <v>326926.68</v>
-      </c>
-      <c r="O166" s="47"/>
-      <c r="P166" s="48"/>
-      <c r="Q166" s="48"/>
-      <c r="R166" s="49"/>
-      <c r="S166" s="54">
-        <v>1.727853162672</v>
-      </c>
-    </row>
-    <row r="167" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A167" s="21" t="s">
+      <c r="B166" s="37">
+        <v>46295</v>
+      </c>
+      <c r="C166" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="D166" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E166" s="45">
+        <v>0.03</v>
+      </c>
+      <c r="F166" s="37">
+        <v>49902</v>
+      </c>
+      <c r="G166" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="H166" s="39">
+        <v>5500</v>
+      </c>
+      <c r="I166" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J166" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="K166" s="39">
+        <v>4829</v>
+      </c>
+      <c r="L166" s="39">
+        <v>2687</v>
+      </c>
+      <c r="M166" s="39">
+        <v>2142</v>
+      </c>
+      <c r="N166" s="40">
+        <v>4177</v>
+      </c>
+      <c r="O166" s="41">
+        <v>95.22</v>
+      </c>
+      <c r="P166" s="40">
+        <v>95.24</v>
+      </c>
+      <c r="Q166" s="40">
+        <v>3.58</v>
+      </c>
+      <c r="R166" s="40">
+        <v>1323</v>
+      </c>
+      <c r="S166" s="44">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="167" spans="1:19">
+      <c r="A167" s="36" t="s">
+        <v>192</v>
+      </c>
+      <c r="B167" s="37">
+        <v>46300</v>
+      </c>
+      <c r="C167" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="D167" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E167" s="35"/>
+      <c r="F167" s="37">
+        <v>46400</v>
+      </c>
+      <c r="G167" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H167" s="39">
+        <v>3000</v>
+      </c>
+      <c r="I167" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J167" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K167" s="39">
+        <v>3311</v>
+      </c>
+      <c r="L167" s="39">
+        <v>2200</v>
+      </c>
+      <c r="M167" s="39">
+        <v>1111</v>
+      </c>
+      <c r="N167" s="40">
+        <v>2426</v>
+      </c>
+      <c r="O167" s="41">
+        <v>99.29773</v>
+      </c>
+      <c r="P167" s="42">
+        <v>99.30095</v>
+      </c>
+      <c r="Q167" s="43">
+        <v>2.586</v>
+      </c>
+      <c r="R167" s="40">
+        <v>574</v>
+      </c>
+      <c r="S167" s="44">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="168" spans="1:19">
+      <c r="A168" s="36" t="s">
+        <v>192</v>
+      </c>
+      <c r="B168" s="37">
+        <v>46300</v>
+      </c>
+      <c r="C168" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="D168" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E168" s="35"/>
+      <c r="F168" s="37">
+        <v>46582</v>
+      </c>
+      <c r="G168" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H168" s="39">
+        <v>3000</v>
+      </c>
+      <c r="I168" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J168" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K168" s="39">
+        <v>5776</v>
+      </c>
+      <c r="L168" s="39">
+        <v>3730</v>
+      </c>
+      <c r="M168" s="39">
+        <v>2046</v>
+      </c>
+      <c r="N168" s="40">
+        <v>2696</v>
+      </c>
+      <c r="O168" s="41">
+        <v>97.81354</v>
+      </c>
+      <c r="P168" s="42">
+        <v>97.81503</v>
+      </c>
+      <c r="Q168" s="43">
+        <v>2.872</v>
+      </c>
+      <c r="R168" s="40">
+        <v>304</v>
+      </c>
+      <c r="S168" s="44">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="169" spans="1:19">
+      <c r="A169" s="36" t="s">
+        <v>193</v>
+      </c>
+      <c r="B169" s="37">
+        <v>46301</v>
+      </c>
+      <c r="C169" s="36" t="s">
+        <v>194</v>
+      </c>
+      <c r="D169" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="E169" s="45">
+        <v>0.03</v>
+      </c>
+      <c r="F169" s="37">
+        <v>47100</v>
+      </c>
+      <c r="G169" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="H169" s="39">
+        <v>6000</v>
+      </c>
+      <c r="I169" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="J169" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="K169" s="39">
+        <v>4869</v>
+      </c>
+      <c r="L169" s="39">
+        <v>2575</v>
+      </c>
+      <c r="M169" s="39">
+        <v>2294</v>
+      </c>
+      <c r="N169" s="40">
+        <v>4526.06</v>
+      </c>
+      <c r="O169" s="41">
+        <v>99.78</v>
+      </c>
+      <c r="P169" s="43">
+        <v>99.792</v>
+      </c>
+      <c r="Q169" s="40">
+        <v>3.1</v>
+      </c>
+      <c r="R169" s="40">
+        <v>1473.94</v>
+      </c>
+      <c r="S169" s="44">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="170" spans="1:19">
+      <c r="A170" s="50" t="s">
+        <v>195</v>
+      </c>
+      <c r="B170" s="48"/>
+      <c r="C170" s="48"/>
+      <c r="D170" s="48"/>
+      <c r="E170" s="48"/>
+      <c r="F170" s="48"/>
+      <c r="G170" s="49"/>
+      <c r="H170" s="52">
+        <v>431000</v>
+      </c>
+      <c r="I170" s="51"/>
+      <c r="J170" s="51"/>
+      <c r="K170" s="52">
+        <v>584027</v>
+      </c>
+      <c r="L170" s="52">
+        <v>344322</v>
+      </c>
+      <c r="M170" s="52">
+        <v>239705</v>
+      </c>
+      <c r="N170" s="53">
+        <v>340751.74</v>
+      </c>
+      <c r="O170" s="47"/>
+      <c r="P170" s="48"/>
+      <c r="Q170" s="48"/>
+      <c r="R170" s="49"/>
+      <c r="S170" s="54">
+        <v>1.713653359481</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A171" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:2">
-      <c r="A168" s="22" t="s">
+    <row r="172" spans="1:2">
+      <c r="A172" s="22" t="s">
         <v>1</v>
-      </c>
-      <c r="B168" s="22" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="169" spans="1:1">
-      <c r="A169" s="22" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2">
-      <c r="A170" s="23" t="s">
-        <v>193</v>
-      </c>
-      <c r="B170" s="26" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="172" spans="1:2">
-      <c r="A172" s="23" t="s">
-        <v>195</v>
       </c>
       <c r="B172" s="22" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="173" spans="1:2">
-      <c r="A173" s="23" t="s">
-        <v>197</v>
-      </c>
-      <c r="B173" s="22" t="s">
-        <v>198</v>
+    <row r="173" spans="1:1">
+      <c r="A173" s="22" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="B174" s="26" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="23" t="s">
         <v>199</v>
       </c>
-      <c r="B174" s="22" t="s">
+      <c r="B176" s="22" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="175" spans="1:2">
-      <c r="A175" s="23" t="s">
+    <row r="177" spans="1:2">
+      <c r="A177" s="23" t="s">
         <v>201</v>
       </c>
-      <c r="B175" s="22" t="s">
+      <c r="B177" s="22" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="176" spans="1:2">
-      <c r="A176" s="24" t="s">
+    <row r="178" spans="1:2">
+      <c r="A178" s="23" t="s">
         <v>203</v>
       </c>
-      <c r="B176" s="22" t="s">
+      <c r="B178" s="22" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="177" spans="1:1">
-      <c r="A177" s="25" t="s">
+    <row r="179" spans="1:2">
+      <c r="A179" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="B179" s="22" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B180" s="22" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1">
+      <c r="A181" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -10370,16 +10614,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A166:G166"/>
-    <mergeCell ref="O166:R166"/>
-    <mergeCell ref="B168:R168"/>
-    <mergeCell ref="A170:A171"/>
-    <mergeCell ref="B170:R171"/>
+    <mergeCell ref="A170:G170"/>
+    <mergeCell ref="O170:R170"/>
     <mergeCell ref="B172:R172"/>
-    <mergeCell ref="B173:R173"/>
-    <mergeCell ref="B174:R174"/>
-    <mergeCell ref="B175:R175"/>
+    <mergeCell ref="A174:A175"/>
+    <mergeCell ref="B174:R175"/>
     <mergeCell ref="B176:R176"/>
+    <mergeCell ref="B177:R177"/>
+    <mergeCell ref="B178:R178"/>
+    <mergeCell ref="B179:R179"/>
+    <mergeCell ref="B180:R180"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-10-12T10:01Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="213" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -723,6 +723,12 @@
   </si>
   <si>
     <t>DE000BU27022</t>
+  </si>
+  <si>
+    <t>98</t>
+  </si>
+  <si>
+    <t>DE000BU0E469</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1166,7 +1172,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S182"/>
+  <dimension ref="A1:S184"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -10568,108 +10574,222 @@
       </c>
     </row>
     <row r="171" spans="1:19">
-      <c r="A171" s="50" t="s">
+      <c r="A171" s="36" t="s">
         <v>197</v>
       </c>
-      <c r="B171" s="48"/>
-      <c r="C171" s="48"/>
-      <c r="D171" s="48"/>
-      <c r="E171" s="48"/>
-      <c r="F171" s="48"/>
-      <c r="G171" s="49"/>
-      <c r="H171" s="52">
-        <v>435000</v>
-      </c>
-      <c r="I171" s="51"/>
-      <c r="J171" s="51"/>
-      <c r="K171" s="52">
-        <v>586746</v>
-      </c>
-      <c r="L171" s="52">
-        <v>346034</v>
-      </c>
-      <c r="M171" s="52">
-        <v>240712</v>
-      </c>
-      <c r="N171" s="53">
-        <v>342663.74</v>
-      </c>
-      <c r="O171" s="47"/>
-      <c r="P171" s="48"/>
-      <c r="Q171" s="48"/>
-      <c r="R171" s="49"/>
-      <c r="S171" s="54">
-        <v>1.711903232013</v>
-      </c>
-    </row>
-    <row r="172" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A172" s="21" t="s">
+      <c r="B171" s="37">
+        <v>46307</v>
+      </c>
+      <c r="C171" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="D171" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E171" s="35"/>
+      <c r="F171" s="37">
+        <v>46491</v>
+      </c>
+      <c r="G171" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H171" s="39">
+        <v>2500</v>
+      </c>
+      <c r="I171" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J171" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K171" s="39">
+        <v>1720</v>
+      </c>
+      <c r="L171" s="39">
+        <v>910</v>
+      </c>
+      <c r="M171" s="39">
+        <v>810</v>
+      </c>
+      <c r="N171" s="40">
+        <v>1495</v>
+      </c>
+      <c r="O171" s="41">
+        <v>98.63862</v>
+      </c>
+      <c r="P171" s="42">
+        <v>98.64502</v>
+      </c>
+      <c r="Q171" s="43">
+        <v>2.717</v>
+      </c>
+      <c r="R171" s="40">
+        <v>1005</v>
+      </c>
+      <c r="S171" s="44">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:19">
+      <c r="A172" s="36" t="s">
+        <v>197</v>
+      </c>
+      <c r="B172" s="37">
+        <v>46307</v>
+      </c>
+      <c r="C172" s="36" t="s">
+        <v>198</v>
+      </c>
+      <c r="D172" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E172" s="35"/>
+      <c r="F172" s="37">
+        <v>46672</v>
+      </c>
+      <c r="G172" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H172" s="39">
+        <v>3500</v>
+      </c>
+      <c r="I172" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="J172" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K172" s="39">
+        <v>4131</v>
+      </c>
+      <c r="L172" s="39">
+        <v>2636</v>
+      </c>
+      <c r="M172" s="39">
+        <v>1495</v>
+      </c>
+      <c r="N172" s="40">
+        <v>2956</v>
+      </c>
+      <c r="O172" s="41">
+        <v>97.10659</v>
+      </c>
+      <c r="P172" s="42">
+        <v>97.11229</v>
+      </c>
+      <c r="Q172" s="43">
+        <v>2.949</v>
+      </c>
+      <c r="R172" s="40">
+        <v>544</v>
+      </c>
+      <c r="S172" s="44">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="173" spans="1:19">
+      <c r="A173" s="50" t="s">
+        <v>199</v>
+      </c>
+      <c r="B173" s="48"/>
+      <c r="C173" s="48"/>
+      <c r="D173" s="48"/>
+      <c r="E173" s="48"/>
+      <c r="F173" s="48"/>
+      <c r="G173" s="49"/>
+      <c r="H173" s="52">
+        <v>441000</v>
+      </c>
+      <c r="I173" s="51"/>
+      <c r="J173" s="51"/>
+      <c r="K173" s="52">
+        <v>592597</v>
+      </c>
+      <c r="L173" s="52">
+        <v>349580</v>
+      </c>
+      <c r="M173" s="52">
+        <v>243017</v>
+      </c>
+      <c r="N173" s="53">
+        <v>347114.74</v>
+      </c>
+      <c r="O173" s="47"/>
+      <c r="P173" s="48"/>
+      <c r="Q173" s="48"/>
+      <c r="R173" s="49"/>
+      <c r="S173" s="54">
+        <v>1.707042357233</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A174" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:2">
-      <c r="A173" s="22" t="s">
+    <row r="175" spans="1:2">
+      <c r="A175" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B173" s="22" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="174" spans="1:1">
-      <c r="A174" s="22" t="s">
+      <c r="B175" s="22" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1">
+      <c r="A176" s="22" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="175" spans="1:2">
-      <c r="A175" s="23" t="s">
-        <v>199</v>
-      </c>
-      <c r="B175" s="26" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="23" t="s">
         <v>201</v>
       </c>
-      <c r="B177" s="22" t="s">
+      <c r="B177" s="26" t="s">
         <v>202</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2">
-      <c r="A178" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="B178" s="22" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="23" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B179" s="22" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="B180" s="22" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="B180" s="22" t="s">
+      <c r="B181" s="22" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="181" spans="1:2">
-      <c r="A181" s="24" t="s">
+    <row r="182" spans="1:2">
+      <c r="A182" s="23" t="s">
         <v>209</v>
       </c>
-      <c r="B181" s="22" t="s">
+      <c r="B182" s="22" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="182" spans="1:1">
-      <c r="A182" s="25" t="s">
+    <row r="183" spans="1:2">
+      <c r="A183" s="24" t="s">
+        <v>211</v>
+      </c>
+      <c r="B183" s="22" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1">
+      <c r="A184" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -10679,16 +10799,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A171:G171"/>
-    <mergeCell ref="O171:R171"/>
-    <mergeCell ref="B173:R173"/>
-    <mergeCell ref="A175:A176"/>
-    <mergeCell ref="B175:R176"/>
-    <mergeCell ref="B177:R177"/>
-    <mergeCell ref="B178:R178"/>
+    <mergeCell ref="A173:G173"/>
+    <mergeCell ref="O173:R173"/>
+    <mergeCell ref="B175:R175"/>
+    <mergeCell ref="A177:A178"/>
+    <mergeCell ref="B177:R178"/>
     <mergeCell ref="B179:R179"/>
     <mergeCell ref="B180:R180"/>
     <mergeCell ref="B181:R181"/>
+    <mergeCell ref="B182:R182"/>
+    <mergeCell ref="B183:R183"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-10-13T10:37Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="213" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="214" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -729,6 +729,9 @@
   </si>
   <si>
     <t>DE000BU0E469</t>
+  </si>
+  <si>
+    <t>99</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1172,7 +1175,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S184"/>
+  <dimension ref="A1:S185"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -10688,108 +10691,167 @@
       </c>
     </row>
     <row r="173" spans="1:19">
-      <c r="A173" s="50" t="s">
+      <c r="A173" s="36" t="s">
         <v>199</v>
       </c>
-      <c r="B173" s="48"/>
-      <c r="C173" s="48"/>
-      <c r="D173" s="48"/>
-      <c r="E173" s="48"/>
-      <c r="F173" s="48"/>
-      <c r="G173" s="49"/>
-      <c r="H173" s="52">
-        <v>441000</v>
-      </c>
-      <c r="I173" s="51"/>
-      <c r="J173" s="51"/>
-      <c r="K173" s="52">
-        <v>592597</v>
-      </c>
-      <c r="L173" s="52">
-        <v>349580</v>
-      </c>
-      <c r="M173" s="52">
-        <v>243017</v>
-      </c>
-      <c r="N173" s="53">
-        <v>347114.74</v>
-      </c>
-      <c r="O173" s="47"/>
-      <c r="P173" s="48"/>
-      <c r="Q173" s="48"/>
-      <c r="R173" s="49"/>
-      <c r="S173" s="54">
-        <v>1.707042357233</v>
-      </c>
-    </row>
-    <row r="174" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A174" s="21" t="s">
+      <c r="B173" s="37">
+        <v>46308</v>
+      </c>
+      <c r="C173" s="36" t="s">
+        <v>166</v>
+      </c>
+      <c r="D173" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="E173" s="45">
+        <v>0.029</v>
+      </c>
+      <c r="F173" s="37">
+        <v>48129</v>
+      </c>
+      <c r="G173" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="H173" s="39">
+        <v>5000</v>
+      </c>
+      <c r="I173" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J173" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="K173" s="39">
+        <v>3607</v>
+      </c>
+      <c r="L173" s="39">
+        <v>2560</v>
+      </c>
+      <c r="M173" s="39">
+        <v>1047</v>
+      </c>
+      <c r="N173" s="40">
+        <v>3352</v>
+      </c>
+      <c r="O173" s="41">
+        <v>98.52</v>
+      </c>
+      <c r="P173" s="40">
+        <v>98.54</v>
+      </c>
+      <c r="Q173" s="40">
+        <v>3.22</v>
+      </c>
+      <c r="R173" s="40">
+        <v>1648</v>
+      </c>
+      <c r="S173" s="44">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:19">
+      <c r="A174" s="50" t="s">
+        <v>200</v>
+      </c>
+      <c r="B174" s="48"/>
+      <c r="C174" s="48"/>
+      <c r="D174" s="48"/>
+      <c r="E174" s="48"/>
+      <c r="F174" s="48"/>
+      <c r="G174" s="49"/>
+      <c r="H174" s="52">
+        <v>446000</v>
+      </c>
+      <c r="I174" s="51"/>
+      <c r="J174" s="51"/>
+      <c r="K174" s="52">
+        <v>596204</v>
+      </c>
+      <c r="L174" s="52">
+        <v>352140</v>
+      </c>
+      <c r="M174" s="52">
+        <v>244064</v>
+      </c>
+      <c r="N174" s="53">
+        <v>350466.74</v>
+      </c>
+      <c r="O174" s="47"/>
+      <c r="P174" s="48"/>
+      <c r="Q174" s="48"/>
+      <c r="R174" s="49"/>
+      <c r="S174" s="54">
+        <v>1.701236368392</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A175" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:2">
-      <c r="A175" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="B175" s="22" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="176" spans="1:1">
+    <row r="176" spans="1:2">
       <c r="A176" s="22" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="177" spans="1:2">
-      <c r="A177" s="23" t="s">
+      <c r="B176" s="22" t="s">
         <v>201</v>
       </c>
-      <c r="B177" s="26" t="s">
+    </row>
+    <row r="177" spans="1:1">
+      <c r="A177" s="22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="23" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="179" spans="1:2">
-      <c r="A179" s="23" t="s">
+      <c r="B178" s="26" t="s">
         <v>203</v>
-      </c>
-      <c r="B179" s="22" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B180" s="22" t="s">
         <v>205</v>
-      </c>
-      <c r="B180" s="22" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="B181" s="22" t="s">
         <v>207</v>
-      </c>
-      <c r="B181" s="22" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="B182" s="22" t="s">
         <v>209</v>
       </c>
-      <c r="B182" s="22" t="s">
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="23" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="183" spans="1:2">
-      <c r="A183" s="24" t="s">
+      <c r="B183" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="B183" s="22" t="s">
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="24" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="184" spans="1:1">
-      <c r="A184" s="25" t="s">
+      <c r="B184" s="22" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1">
+      <c r="A185" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -10799,16 +10861,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A173:G173"/>
-    <mergeCell ref="O173:R173"/>
-    <mergeCell ref="B175:R175"/>
-    <mergeCell ref="A177:A178"/>
-    <mergeCell ref="B177:R178"/>
-    <mergeCell ref="B179:R179"/>
+    <mergeCell ref="A174:G174"/>
+    <mergeCell ref="O174:R174"/>
+    <mergeCell ref="B176:R176"/>
+    <mergeCell ref="A178:A179"/>
+    <mergeCell ref="B178:R179"/>
     <mergeCell ref="B180:R180"/>
     <mergeCell ref="B181:R181"/>
     <mergeCell ref="B182:R182"/>
     <mergeCell ref="B183:R183"/>
+    <mergeCell ref="B184:R184"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-10-14T09:49Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="214" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="215" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -732,6 +732,9 @@
   </si>
   <si>
     <t>99</t>
+  </si>
+  <si>
+    <t>100</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1175,7 +1178,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S185"/>
+  <dimension ref="A1:S187"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -10750,108 +10753,226 @@
       </c>
     </row>
     <row r="174" spans="1:19">
-      <c r="A174" s="50" t="s">
+      <c r="A174" s="36" t="s">
         <v>200</v>
       </c>
-      <c r="B174" s="48"/>
-      <c r="C174" s="48"/>
-      <c r="D174" s="48"/>
-      <c r="E174" s="48"/>
-      <c r="F174" s="48"/>
-      <c r="G174" s="49"/>
-      <c r="H174" s="52">
-        <v>446000</v>
-      </c>
-      <c r="I174" s="51"/>
-      <c r="J174" s="51"/>
-      <c r="K174" s="52">
-        <v>596204</v>
-      </c>
-      <c r="L174" s="52">
-        <v>352140</v>
-      </c>
-      <c r="M174" s="52">
-        <v>244064</v>
-      </c>
-      <c r="N174" s="53">
-        <v>350466.74</v>
-      </c>
-      <c r="O174" s="47"/>
-      <c r="P174" s="48"/>
-      <c r="Q174" s="48"/>
-      <c r="R174" s="49"/>
-      <c r="S174" s="54">
-        <v>1.701236368392</v>
-      </c>
-    </row>
-    <row r="175" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A175" s="21" t="s">
+      <c r="B174" s="37">
+        <v>46309</v>
+      </c>
+      <c r="C174" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="D174" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E174" s="45">
+        <v>0.034</v>
+      </c>
+      <c r="F174" s="37">
+        <v>53827</v>
+      </c>
+      <c r="G174" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="H174" s="39">
+        <v>1500</v>
+      </c>
+      <c r="I174" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J174" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K174" s="39">
+        <v>2802</v>
+      </c>
+      <c r="L174" s="39">
+        <v>770</v>
+      </c>
+      <c r="M174" s="39">
+        <v>2032</v>
+      </c>
+      <c r="N174" s="40">
+        <v>1141.4</v>
+      </c>
+      <c r="O174" s="41">
+        <v>94.3</v>
+      </c>
+      <c r="P174" s="40">
+        <v>94.3</v>
+      </c>
+      <c r="Q174" s="40">
+        <v>3.8</v>
+      </c>
+      <c r="R174" s="40">
+        <v>358.6</v>
+      </c>
+      <c r="S174" s="44">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="175" spans="1:19">
+      <c r="A175" s="36" t="s">
+        <v>200</v>
+      </c>
+      <c r="B175" s="37">
+        <v>46309</v>
+      </c>
+      <c r="C175" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="D175" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E175" s="45">
+        <v>0.029</v>
+      </c>
+      <c r="F175" s="37">
+        <v>57207</v>
+      </c>
+      <c r="G175" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="H175" s="39">
+        <v>1000</v>
+      </c>
+      <c r="I175" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J175" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K175" s="39">
+        <v>1058</v>
+      </c>
+      <c r="L175" s="39">
+        <v>497</v>
+      </c>
+      <c r="M175" s="39">
+        <v>561</v>
+      </c>
+      <c r="N175" s="40">
+        <v>747.39</v>
+      </c>
+      <c r="O175" s="41">
+        <v>83.98</v>
+      </c>
+      <c r="P175" s="40">
+        <v>84.04</v>
+      </c>
+      <c r="Q175" s="40">
+        <v>3.8</v>
+      </c>
+      <c r="R175" s="40">
+        <v>252.61</v>
+      </c>
+      <c r="S175" s="44">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="176" spans="1:19">
+      <c r="A176" s="50" t="s">
+        <v>201</v>
+      </c>
+      <c r="B176" s="48"/>
+      <c r="C176" s="48"/>
+      <c r="D176" s="48"/>
+      <c r="E176" s="48"/>
+      <c r="F176" s="48"/>
+      <c r="G176" s="49"/>
+      <c r="H176" s="52">
+        <v>448500</v>
+      </c>
+      <c r="I176" s="51"/>
+      <c r="J176" s="51"/>
+      <c r="K176" s="52">
+        <v>600064</v>
+      </c>
+      <c r="L176" s="52">
+        <v>353407</v>
+      </c>
+      <c r="M176" s="52">
+        <v>246657</v>
+      </c>
+      <c r="N176" s="53">
+        <v>352355.53</v>
+      </c>
+      <c r="O176" s="47"/>
+      <c r="P176" s="48"/>
+      <c r="Q176" s="48"/>
+      <c r="R176" s="49"/>
+      <c r="S176" s="54">
+        <v>1.703184876933</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A177" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:2">
-      <c r="A176" s="22" t="s">
+    <row r="178" spans="1:2">
+      <c r="A178" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B176" s="22" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="177" spans="1:1">
-      <c r="A177" s="22" t="s">
+      <c r="B178" s="22" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1">
+      <c r="A179" s="22" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2">
-      <c r="A178" s="23" t="s">
-        <v>202</v>
-      </c>
-      <c r="B178" s="26" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="B180" s="26" t="s">
         <v>204</v>
-      </c>
-      <c r="B180" s="22" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2">
-      <c r="A181" s="23" t="s">
-        <v>206</v>
-      </c>
-      <c r="B181" s="22" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="23" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B182" s="22" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="B183" s="22" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B184" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="B183" s="22" t="s">
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="23" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="184" spans="1:2">
-      <c r="A184" s="24" t="s">
+      <c r="B185" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="B184" s="22" t="s">
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="24" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="185" spans="1:1">
-      <c r="A185" s="25" t="s">
+      <c r="B186" s="22" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1">
+      <c r="A187" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -10861,16 +10982,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A174:G174"/>
-    <mergeCell ref="O174:R174"/>
-    <mergeCell ref="B176:R176"/>
-    <mergeCell ref="A178:A179"/>
-    <mergeCell ref="B178:R179"/>
-    <mergeCell ref="B180:R180"/>
-    <mergeCell ref="B181:R181"/>
+    <mergeCell ref="A176:G176"/>
+    <mergeCell ref="O176:R176"/>
+    <mergeCell ref="B178:R178"/>
+    <mergeCell ref="A180:A181"/>
+    <mergeCell ref="B180:R181"/>
     <mergeCell ref="B182:R182"/>
     <mergeCell ref="B183:R183"/>
     <mergeCell ref="B184:R184"/>
+    <mergeCell ref="B185:R185"/>
+    <mergeCell ref="B186:R186"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-10-19T15:55Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="215" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="216" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -735,6 +735,9 @@
   </si>
   <si>
     <t>100</t>
+  </si>
+  <si>
+    <t>101</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1178,7 +1181,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S187"/>
+  <dimension ref="A1:S189"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -10871,108 +10874,222 @@
       </c>
     </row>
     <row r="176" spans="1:19">
-      <c r="A176" s="50" t="s">
+      <c r="A176" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="B176" s="48"/>
-      <c r="C176" s="48"/>
-      <c r="D176" s="48"/>
-      <c r="E176" s="48"/>
-      <c r="F176" s="48"/>
-      <c r="G176" s="49"/>
-      <c r="H176" s="52">
-        <v>448500</v>
-      </c>
-      <c r="I176" s="51"/>
-      <c r="J176" s="51"/>
-      <c r="K176" s="52">
-        <v>600064</v>
-      </c>
-      <c r="L176" s="52">
-        <v>353407</v>
-      </c>
-      <c r="M176" s="52">
-        <v>246657</v>
-      </c>
-      <c r="N176" s="53">
-        <v>352355.53</v>
-      </c>
-      <c r="O176" s="47"/>
-      <c r="P176" s="48"/>
-      <c r="Q176" s="48"/>
-      <c r="R176" s="49"/>
-      <c r="S176" s="54">
-        <v>1.703184876933</v>
-      </c>
-    </row>
-    <row r="177" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A177" s="21" t="s">
+      <c r="B176" s="37">
+        <v>46314</v>
+      </c>
+      <c r="C176" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D176" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E176" s="35"/>
+      <c r="F176" s="37">
+        <v>46463</v>
+      </c>
+      <c r="G176" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H176" s="39">
+        <v>3000</v>
+      </c>
+      <c r="I176" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J176" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K176" s="39">
+        <v>1850</v>
+      </c>
+      <c r="L176" s="39">
+        <v>1495</v>
+      </c>
+      <c r="M176" s="39">
+        <v>355</v>
+      </c>
+      <c r="N176" s="40">
+        <v>1550</v>
+      </c>
+      <c r="O176" s="41">
+        <v>98.90553</v>
+      </c>
+      <c r="P176" s="42">
+        <v>98.90992</v>
+      </c>
+      <c r="Q176" s="43">
+        <v>2.699</v>
+      </c>
+      <c r="R176" s="40">
+        <v>1450</v>
+      </c>
+      <c r="S176" s="44">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="177" spans="1:19">
+      <c r="A177" s="36" t="s">
+        <v>201</v>
+      </c>
+      <c r="B177" s="37">
+        <v>46314</v>
+      </c>
+      <c r="C177" s="36" t="s">
+        <v>185</v>
+      </c>
+      <c r="D177" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E177" s="35"/>
+      <c r="F177" s="37">
+        <v>46645</v>
+      </c>
+      <c r="G177" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H177" s="39">
+        <v>2000</v>
+      </c>
+      <c r="I177" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J177" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K177" s="39">
+        <v>2076</v>
+      </c>
+      <c r="L177" s="39">
+        <v>1821</v>
+      </c>
+      <c r="M177" s="39">
+        <v>255</v>
+      </c>
+      <c r="N177" s="40">
+        <v>1351</v>
+      </c>
+      <c r="O177" s="41">
+        <v>97.37134</v>
+      </c>
+      <c r="P177" s="42">
+        <v>97.37914</v>
+      </c>
+      <c r="Q177" s="43">
+        <v>2.945</v>
+      </c>
+      <c r="R177" s="40">
+        <v>649</v>
+      </c>
+      <c r="S177" s="44">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="178" spans="1:19">
+      <c r="A178" s="50" t="s">
+        <v>202</v>
+      </c>
+      <c r="B178" s="48"/>
+      <c r="C178" s="48"/>
+      <c r="D178" s="48"/>
+      <c r="E178" s="48"/>
+      <c r="F178" s="48"/>
+      <c r="G178" s="49"/>
+      <c r="H178" s="52">
+        <v>453500</v>
+      </c>
+      <c r="I178" s="51"/>
+      <c r="J178" s="51"/>
+      <c r="K178" s="52">
+        <v>603990</v>
+      </c>
+      <c r="L178" s="52">
+        <v>356723</v>
+      </c>
+      <c r="M178" s="52">
+        <v>247267</v>
+      </c>
+      <c r="N178" s="53">
+        <v>355256.53</v>
+      </c>
+      <c r="O178" s="47"/>
+      <c r="P178" s="48"/>
+      <c r="Q178" s="48"/>
+      <c r="R178" s="49"/>
+      <c r="S178" s="54">
+        <v>1.700216770118</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A179" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:2">
-      <c r="A178" s="22" t="s">
+    <row r="180" spans="1:2">
+      <c r="A180" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B178" s="22" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="179" spans="1:1">
-      <c r="A179" s="22" t="s">
+      <c r="B180" s="22" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1">
+      <c r="A181" s="22" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2">
-      <c r="A180" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="B180" s="26" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B182" s="26" t="s">
         <v>205</v>
-      </c>
-      <c r="B182" s="22" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2">
-      <c r="A183" s="23" t="s">
-        <v>207</v>
-      </c>
-      <c r="B183" s="22" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="23" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B184" s="22" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="B185" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="B186" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="B185" s="22" t="s">
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="23" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="186" spans="1:2">
-      <c r="A186" s="24" t="s">
+      <c r="B187" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="B186" s="22" t="s">
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="24" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="187" spans="1:1">
-      <c r="A187" s="25" t="s">
+      <c r="B188" s="22" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1">
+      <c r="A189" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -10982,16 +11099,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A176:G176"/>
-    <mergeCell ref="O176:R176"/>
-    <mergeCell ref="B178:R178"/>
-    <mergeCell ref="A180:A181"/>
-    <mergeCell ref="B180:R181"/>
-    <mergeCell ref="B182:R182"/>
-    <mergeCell ref="B183:R183"/>
+    <mergeCell ref="A178:G178"/>
+    <mergeCell ref="O178:R178"/>
+    <mergeCell ref="B180:R180"/>
+    <mergeCell ref="A182:A183"/>
+    <mergeCell ref="B182:R183"/>
     <mergeCell ref="B184:R184"/>
     <mergeCell ref="B185:R185"/>
     <mergeCell ref="B186:R186"/>
+    <mergeCell ref="B187:R187"/>
+    <mergeCell ref="B188:R188"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-10-20T13:00Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="216" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -738,6 +738,9 @@
   </si>
   <si>
     <t>101</t>
+  </si>
+  <si>
+    <t>102</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1181,7 +1184,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S189"/>
+  <dimension ref="A1:S191"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -10988,108 +10991,226 @@
       </c>
     </row>
     <row r="178" spans="1:19">
-      <c r="A178" s="50" t="s">
+      <c r="A178" s="36" t="s">
         <v>202</v>
       </c>
-      <c r="B178" s="48"/>
-      <c r="C178" s="48"/>
-      <c r="D178" s="48"/>
-      <c r="E178" s="48"/>
-      <c r="F178" s="48"/>
-      <c r="G178" s="49"/>
-      <c r="H178" s="52">
-        <v>453500</v>
-      </c>
-      <c r="I178" s="51"/>
-      <c r="J178" s="51"/>
-      <c r="K178" s="52">
-        <v>603990</v>
-      </c>
-      <c r="L178" s="52">
-        <v>356723</v>
-      </c>
-      <c r="M178" s="52">
-        <v>247267</v>
-      </c>
-      <c r="N178" s="53">
-        <v>355256.53</v>
-      </c>
-      <c r="O178" s="47"/>
-      <c r="P178" s="48"/>
-      <c r="Q178" s="48"/>
-      <c r="R178" s="49"/>
-      <c r="S178" s="54">
-        <v>1.700216770118</v>
-      </c>
-    </row>
-    <row r="179" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A179" s="21" t="s">
+      <c r="B178" s="37">
+        <v>46315</v>
+      </c>
+      <c r="C178" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="D178" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="E178" s="45">
+        <v>0.018</v>
+      </c>
+      <c r="F178" s="37">
+        <v>56111</v>
+      </c>
+      <c r="G178" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="H178" s="39">
+        <v>500</v>
+      </c>
+      <c r="I178" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J178" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K178" s="39">
+        <v>803</v>
+      </c>
+      <c r="L178" s="39">
+        <v>342</v>
+      </c>
+      <c r="M178" s="39">
+        <v>461</v>
+      </c>
+      <c r="N178" s="40">
+        <v>498</v>
+      </c>
+      <c r="O178" s="41">
+        <v>66.89</v>
+      </c>
+      <c r="P178" s="40">
+        <v>66.89</v>
+      </c>
+      <c r="Q178" s="40">
+        <v>3.79</v>
+      </c>
+      <c r="R178" s="40">
+        <v>2</v>
+      </c>
+      <c r="S178" s="44">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="179" spans="1:19">
+      <c r="A179" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="B179" s="37">
+        <v>46315</v>
+      </c>
+      <c r="C179" s="36" t="s">
+        <v>129</v>
+      </c>
+      <c r="D179" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="E179" s="45">
+        <v>0.021</v>
+      </c>
+      <c r="F179" s="37">
+        <v>47220</v>
+      </c>
+      <c r="G179" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="H179" s="39">
+        <v>500</v>
+      </c>
+      <c r="I179" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J179" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="K179" s="39">
+        <v>966</v>
+      </c>
+      <c r="L179" s="39">
+        <v>532</v>
+      </c>
+      <c r="M179" s="39">
+        <v>434</v>
+      </c>
+      <c r="N179" s="40">
+        <v>494</v>
+      </c>
+      <c r="O179" s="41">
+        <v>97.69</v>
+      </c>
+      <c r="P179" s="40">
+        <v>97.69</v>
+      </c>
+      <c r="Q179" s="40">
+        <v>3.08</v>
+      </c>
+      <c r="R179" s="40">
+        <v>6</v>
+      </c>
+      <c r="S179" s="44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="180" spans="1:19">
+      <c r="A180" s="50" t="s">
+        <v>203</v>
+      </c>
+      <c r="B180" s="48"/>
+      <c r="C180" s="48"/>
+      <c r="D180" s="48"/>
+      <c r="E180" s="48"/>
+      <c r="F180" s="48"/>
+      <c r="G180" s="49"/>
+      <c r="H180" s="52">
+        <v>454500</v>
+      </c>
+      <c r="I180" s="51"/>
+      <c r="J180" s="51"/>
+      <c r="K180" s="52">
+        <v>605759</v>
+      </c>
+      <c r="L180" s="52">
+        <v>357597</v>
+      </c>
+      <c r="M180" s="52">
+        <v>248162</v>
+      </c>
+      <c r="N180" s="53">
+        <v>356248.53</v>
+      </c>
+      <c r="O180" s="47"/>
+      <c r="P180" s="48"/>
+      <c r="Q180" s="48"/>
+      <c r="R180" s="49"/>
+      <c r="S180" s="54">
+        <v>1.700492378172</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A181" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:2">
-      <c r="A180" s="22" t="s">
+    <row r="182" spans="1:2">
+      <c r="A182" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B180" s="22" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="181" spans="1:1">
-      <c r="A181" s="22" t="s">
+      <c r="B182" s="22" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1">
+      <c r="A183" s="22" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2">
-      <c r="A182" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="B182" s="26" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="B184" s="26" t="s">
         <v>206</v>
-      </c>
-      <c r="B184" s="22" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2">
-      <c r="A185" s="23" t="s">
-        <v>208</v>
-      </c>
-      <c r="B185" s="22" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="23" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B186" s="22" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B187" s="22" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="23" t="s">
+        <v>211</v>
+      </c>
+      <c r="B188" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="B187" s="22" t="s">
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="23" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="188" spans="1:2">
-      <c r="A188" s="24" t="s">
+      <c r="B189" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="B188" s="22" t="s">
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="24" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="189" spans="1:1">
-      <c r="A189" s="25" t="s">
+      <c r="B190" s="22" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1">
+      <c r="A191" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -11099,16 +11220,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A178:G178"/>
-    <mergeCell ref="O178:R178"/>
-    <mergeCell ref="B180:R180"/>
-    <mergeCell ref="A182:A183"/>
-    <mergeCell ref="B182:R183"/>
-    <mergeCell ref="B184:R184"/>
-    <mergeCell ref="B185:R185"/>
+    <mergeCell ref="A180:G180"/>
+    <mergeCell ref="O180:R180"/>
+    <mergeCell ref="B182:R182"/>
+    <mergeCell ref="A184:A185"/>
+    <mergeCell ref="B184:R185"/>
     <mergeCell ref="B186:R186"/>
     <mergeCell ref="B187:R187"/>
     <mergeCell ref="B188:R188"/>
+    <mergeCell ref="B189:R189"/>
+    <mergeCell ref="B190:R190"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-10-27T12:08Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -741,6 +741,9 @@
   </si>
   <si>
     <t>102</t>
+  </si>
+  <si>
+    <t>103</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1184,7 +1187,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S191"/>
+  <dimension ref="A1:S192"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -11109,108 +11112,167 @@
       </c>
     </row>
     <row r="180" spans="1:19">
-      <c r="A180" s="50" t="s">
+      <c r="A180" s="36" t="s">
         <v>203</v>
       </c>
-      <c r="B180" s="48"/>
-      <c r="C180" s="48"/>
-      <c r="D180" s="48"/>
-      <c r="E180" s="48"/>
-      <c r="F180" s="48"/>
-      <c r="G180" s="49"/>
-      <c r="H180" s="52">
-        <v>454500</v>
-      </c>
-      <c r="I180" s="51"/>
-      <c r="J180" s="51"/>
-      <c r="K180" s="52">
-        <v>605759</v>
-      </c>
-      <c r="L180" s="52">
-        <v>357597</v>
-      </c>
-      <c r="M180" s="52">
-        <v>248162</v>
-      </c>
-      <c r="N180" s="53">
-        <v>356248.53</v>
-      </c>
-      <c r="O180" s="47"/>
-      <c r="P180" s="48"/>
-      <c r="Q180" s="48"/>
-      <c r="R180" s="49"/>
-      <c r="S180" s="54">
-        <v>1.700492378172</v>
-      </c>
-    </row>
-    <row r="181" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A181" s="21" t="s">
+      <c r="B180" s="37">
+        <v>46322</v>
+      </c>
+      <c r="C180" s="36" t="s">
+        <v>194</v>
+      </c>
+      <c r="D180" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="E180" s="45">
+        <v>0.03</v>
+      </c>
+      <c r="F180" s="37">
+        <v>47100</v>
+      </c>
+      <c r="G180" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="H180" s="39">
+        <v>5000</v>
+      </c>
+      <c r="I180" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J180" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="K180" s="39">
+        <v>5047</v>
+      </c>
+      <c r="L180" s="39">
+        <v>3623</v>
+      </c>
+      <c r="M180" s="39">
+        <v>1424</v>
+      </c>
+      <c r="N180" s="40">
+        <v>3790.36</v>
+      </c>
+      <c r="O180" s="41">
+        <v>99.825</v>
+      </c>
+      <c r="P180" s="43">
+        <v>99.828</v>
+      </c>
+      <c r="Q180" s="40">
+        <v>3.08</v>
+      </c>
+      <c r="R180" s="40">
+        <v>1209.64</v>
+      </c>
+      <c r="S180" s="44">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="181" spans="1:19">
+      <c r="A181" s="50" t="s">
+        <v>204</v>
+      </c>
+      <c r="B181" s="48"/>
+      <c r="C181" s="48"/>
+      <c r="D181" s="48"/>
+      <c r="E181" s="48"/>
+      <c r="F181" s="48"/>
+      <c r="G181" s="49"/>
+      <c r="H181" s="52">
+        <v>459500</v>
+      </c>
+      <c r="I181" s="51"/>
+      <c r="J181" s="51"/>
+      <c r="K181" s="52">
+        <v>610806</v>
+      </c>
+      <c r="L181" s="52">
+        <v>361220</v>
+      </c>
+      <c r="M181" s="52">
+        <v>249586</v>
+      </c>
+      <c r="N181" s="53">
+        <v>360038.89</v>
+      </c>
+      <c r="O181" s="47"/>
+      <c r="P181" s="48"/>
+      <c r="Q181" s="48"/>
+      <c r="R181" s="49"/>
+      <c r="S181" s="54">
+        <v>1.696276138391</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A182" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:2">
-      <c r="A182" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="B182" s="22" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="183" spans="1:1">
+    <row r="183" spans="1:2">
       <c r="A183" s="22" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="184" spans="1:2">
-      <c r="A184" s="23" t="s">
+      <c r="B183" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="B184" s="26" t="s">
+    </row>
+    <row r="184" spans="1:1">
+      <c r="A184" s="22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="23" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="186" spans="1:2">
-      <c r="A186" s="23" t="s">
+      <c r="B185" s="26" t="s">
         <v>207</v>
-      </c>
-      <c r="B186" s="22" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="B187" s="22" t="s">
         <v>209</v>
-      </c>
-      <c r="B187" s="22" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="B188" s="22" t="s">
         <v>211</v>
-      </c>
-      <c r="B188" s="22" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="B189" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="B189" s="22" t="s">
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="23" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="190" spans="1:2">
-      <c r="A190" s="24" t="s">
+      <c r="B190" s="22" t="s">
         <v>215</v>
       </c>
-      <c r="B190" s="22" t="s">
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="24" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="191" spans="1:1">
-      <c r="A191" s="25" t="s">
+      <c r="B191" s="22" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1">
+      <c r="A192" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -11220,16 +11282,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A180:G180"/>
-    <mergeCell ref="O180:R180"/>
-    <mergeCell ref="B182:R182"/>
-    <mergeCell ref="A184:A185"/>
-    <mergeCell ref="B184:R185"/>
-    <mergeCell ref="B186:R186"/>
+    <mergeCell ref="A181:G181"/>
+    <mergeCell ref="O181:R181"/>
+    <mergeCell ref="B183:R183"/>
+    <mergeCell ref="A185:A186"/>
+    <mergeCell ref="B185:R186"/>
     <mergeCell ref="B187:R187"/>
     <mergeCell ref="B188:R188"/>
     <mergeCell ref="B189:R189"/>
     <mergeCell ref="B190:R190"/>
+    <mergeCell ref="B191:R191"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
data(eur): daily refresh 2026-10-28T13:04Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="219" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -744,6 +744,9 @@
   </si>
   <si>
     <t>103</t>
+  </si>
+  <si>
+    <t>104</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1187,7 +1190,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S192"/>
+  <dimension ref="A1:S193"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -11171,108 +11174,167 @@
       </c>
     </row>
     <row r="181" spans="1:19">
-      <c r="A181" s="50" t="s">
+      <c r="A181" s="36" t="s">
         <v>204</v>
       </c>
-      <c r="B181" s="48"/>
-      <c r="C181" s="48"/>
-      <c r="D181" s="48"/>
-      <c r="E181" s="48"/>
-      <c r="F181" s="48"/>
-      <c r="G181" s="49"/>
-      <c r="H181" s="52">
-        <v>459500</v>
-      </c>
-      <c r="I181" s="51"/>
-      <c r="J181" s="51"/>
-      <c r="K181" s="52">
-        <v>610806</v>
-      </c>
-      <c r="L181" s="52">
-        <v>361220</v>
-      </c>
-      <c r="M181" s="52">
-        <v>249586</v>
-      </c>
-      <c r="N181" s="53">
-        <v>360038.89</v>
-      </c>
-      <c r="O181" s="47"/>
-      <c r="P181" s="48"/>
-      <c r="Q181" s="48"/>
-      <c r="R181" s="49"/>
-      <c r="S181" s="54">
-        <v>1.696276138391</v>
-      </c>
-    </row>
-    <row r="182" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A182" s="21" t="s">
+      <c r="B181" s="37">
+        <v>46323</v>
+      </c>
+      <c r="C181" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="D181" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E181" s="45">
+        <v>0.03</v>
+      </c>
+      <c r="F181" s="37">
+        <v>49902</v>
+      </c>
+      <c r="G181" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="H181" s="39">
+        <v>5500</v>
+      </c>
+      <c r="I181" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J181" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="K181" s="39">
+        <v>4460</v>
+      </c>
+      <c r="L181" s="39">
+        <v>3143</v>
+      </c>
+      <c r="M181" s="39">
+        <v>1317</v>
+      </c>
+      <c r="N181" s="40">
+        <v>3890</v>
+      </c>
+      <c r="O181" s="41">
+        <v>96.93</v>
+      </c>
+      <c r="P181" s="40">
+        <v>96.95</v>
+      </c>
+      <c r="Q181" s="40">
+        <v>3.37</v>
+      </c>
+      <c r="R181" s="40">
+        <v>1610</v>
+      </c>
+      <c r="S181" s="44">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:19">
+      <c r="A182" s="50" t="s">
+        <v>205</v>
+      </c>
+      <c r="B182" s="48"/>
+      <c r="C182" s="48"/>
+      <c r="D182" s="48"/>
+      <c r="E182" s="48"/>
+      <c r="F182" s="48"/>
+      <c r="G182" s="49"/>
+      <c r="H182" s="52">
+        <v>465000</v>
+      </c>
+      <c r="I182" s="51"/>
+      <c r="J182" s="51"/>
+      <c r="K182" s="52">
+        <v>615266</v>
+      </c>
+      <c r="L182" s="52">
+        <v>364363</v>
+      </c>
+      <c r="M182" s="52">
+        <v>250903</v>
+      </c>
+      <c r="N182" s="53">
+        <v>363928.89</v>
+      </c>
+      <c r="O182" s="47"/>
+      <c r="P182" s="48"/>
+      <c r="Q182" s="48"/>
+      <c r="R182" s="49"/>
+      <c r="S182" s="54">
+        <v>1.689902601576</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A183" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:2">
-      <c r="A183" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="B183" s="22" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="184" spans="1:1">
+    <row r="184" spans="1:2">
       <c r="A184" s="22" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="185" spans="1:2">
-      <c r="A185" s="23" t="s">
+      <c r="B184" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="B185" s="26" t="s">
+    </row>
+    <row r="185" spans="1:1">
+      <c r="A185" s="22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="23" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="187" spans="1:2">
-      <c r="A187" s="23" t="s">
+      <c r="B186" s="26" t="s">
         <v>208</v>
-      </c>
-      <c r="B187" s="22" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B188" s="22" t="s">
         <v>210</v>
-      </c>
-      <c r="B188" s="22" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="23" t="s">
+        <v>211</v>
+      </c>
+      <c r="B189" s="22" t="s">
         <v>212</v>
-      </c>
-      <c r="B189" s="22" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="B190" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="B190" s="22" t="s">
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="23" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="191" spans="1:2">
-      <c r="A191" s="24" t="s">
+      <c r="B191" s="22" t="s">
         <v>216</v>
       </c>
-      <c r="B191" s="22" t="s">
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="24" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="192" spans="1:1">
-      <c r="A192" s="25" t="s">
+      <c r="B192" s="22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1">
+      <c r="A193" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -11282,16 +11344,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A181:G181"/>
-    <mergeCell ref="O181:R181"/>
-    <mergeCell ref="B183:R183"/>
-    <mergeCell ref="A185:A186"/>
-    <mergeCell ref="B185:R186"/>
-    <mergeCell ref="B187:R187"/>
+    <mergeCell ref="A182:G182"/>
+    <mergeCell ref="O182:R182"/>
+    <mergeCell ref="B184:R184"/>
+    <mergeCell ref="A186:A187"/>
+    <mergeCell ref="B186:R187"/>
     <mergeCell ref="B188:R188"/>
     <mergeCell ref="B189:R189"/>
     <mergeCell ref="B190:R190"/>
     <mergeCell ref="B191:R191"/>
+    <mergeCell ref="B192:R192"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>